<commit_message>
added text,telephone and tax code validation
</commit_message>
<xml_diff>
--- a/DQ_Rule_Catalog.xlsx
+++ b/DQ_Rule_Catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vivek/Documents/Data Science Projects/data-quality-solution/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B5507D-6A44-5E45-9735-255A0514B479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E99D7EE-E868-A24C-A4F1-0C0C3B31501C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="125">
   <si>
     <t>RULE_ID</t>
   </si>
@@ -392,6 +392,9 @@
   </si>
   <si>
     <t>Vendor Master</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
 </sst>
 </file>
@@ -410,7 +413,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -420,6 +423,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -435,12 +444,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,12 +486,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="VendorDQRuleCatalog" displayName="VendorDQRuleCatalog" ref="A1:K26" totalsRowShown="0">
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="RULE_ID"/>
-    <tableColumn id="11" xr3:uid="{159DBD3F-780B-E24F-85B1-FA3C07D7B7A2}" name="WORKSTREAM" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{159DBD3F-780B-E24F-85B1-FA3C07D7B7A2}" name="WORKSTREAM" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="OBJECT"/>
     <tableColumn id="10" xr3:uid="{FF065E68-683E-1641-840C-780062416B5E}" name="KEY" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FIELD"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="DQ_DIMENSION"/>
-    <tableColumn id="9" xr3:uid="{C0CE0C18-9332-2A45-8540-8D00F9CEAD27}" name="RULE_CLASS" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{C0CE0C18-9332-2A45-8540-8D00F9CEAD27}" name="RULE_CLASS" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="RULE_TYPE"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="RULE_DESCRIPTION"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="ISSUE"/>
@@ -747,7 +759,7 @@
       <c r="D2" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -782,7 +794,7 @@
       <c r="D3" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F3" s="2" t="s">
@@ -817,7 +829,7 @@
       <c r="D4" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="2" t="s">
@@ -852,7 +864,7 @@
       <c r="D5" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>24</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -887,7 +899,7 @@
       <c r="D6" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -922,7 +934,7 @@
       <c r="D7" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -957,7 +969,7 @@
       <c r="D8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>36</v>
       </c>
       <c r="F8" s="2" t="s">
@@ -1342,7 +1354,7 @@
       <c r="D19" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F19" s="2" t="s">
@@ -1377,7 +1389,7 @@
       <c r="D20" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F20" s="2" t="s">
@@ -1431,7 +1443,7 @@
         <v>92</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>14</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="56" customHeight="1">
@@ -1466,7 +1478,7 @@
         <v>96</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>14</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="56" customHeight="1">

</xml_diff>